<commit_message>
Updated URP scene to use Renderer Feature instead of Camera Stacking for improved performance.
</commit_message>
<xml_diff>
--- a/Results/Summary.xlsx
+++ b/Results/Summary.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Source\unity-birp-vs-urp-performance\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D39E519E-2771-4D13-BEBF-5292969A820B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12336A37-C177-47B0-A778-6CED643F60F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="51420" windowHeight="21100" xr2:uid="{063CB107-2C1C-4A1E-A4C3-45183028293E}"/>
+    <workbookView xWindow="24910" yWindow="0" windowWidth="25780" windowHeight="20970" xr2:uid="{063CB107-2C1C-4A1E-A4C3-45183028293E}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="20">
   <si>
     <t>GTX 1650</t>
   </si>
@@ -60,9 +60,6 @@
   </si>
   <si>
     <t>RTX 4090</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> URP</t>
   </si>
   <si>
     <t>Frame</t>
@@ -317,6 +314,44 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-4C57-4F42-9222-F063B02C7613}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000002-3F41-4E91-9E7D-15E090A83700}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln>
@@ -326,7 +361,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000002-4C57-4F42-9222-F063B02C7613}"/>
+                <c16:uniqueId val="{00000003-3F41-4E91-9E7D-15E090A83700}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -363,10 +398,10 @@
                   <c:v>9.65</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.42</c:v>
+                  <c:v>8.41</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11.95</c:v>
+                  <c:v>11.43</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -715,10 +750,10 @@
                   <c:v>6.65</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>5.13</c:v>
+                  <c:v>4.42</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>5.66</c:v>
+                  <c:v>5.0999999999999996</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1020,6 +1055,25 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-AB4D-44D7-B016-AC3468EBAAD8}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln>
@@ -1029,7 +1083,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-AB4D-44D7-B016-AC3468EBAAD8}"/>
+                <c16:uniqueId val="{00000002-126C-4138-BE77-E07B0BEA9419}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1066,10 +1120,10 @@
                   <c:v>103.5</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>105.3</c:v>
+                  <c:v>117.2</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>83.5</c:v>
+                  <c:v>82.4</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1389,7 +1443,7 @@
                   <c:v>RTX 4090 DX11 URP</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>RTX 4090 DX12  URP</c:v>
+                  <c:v>RTX 4090 DX12 URP</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1407,10 +1461,10 @@
                   <c:v>1.1599999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1200000000000001</c:v>
+                  <c:v>0.92</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.61</c:v>
+                  <c:v>1.36</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -1702,6 +1756,25 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-608E-4F9B-A5AD-B7018EE3A269}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln>
@@ -1711,7 +1784,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-608E-4F9B-A5AD-B7018EE3A269}"/>
+                <c16:uniqueId val="{00000002-B20F-4335-A212-E31D73E00D61}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -1730,7 +1803,7 @@
                   <c:v>RTX 4090 DX11 URP</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>RTX 4090 DX12  URP</c:v>
+                  <c:v>RTX 4090 DX12 URP</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -1748,10 +1821,10 @@
                   <c:v>0.94</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.77</c:v>
+                  <c:v>0.64</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.83</c:v>
+                  <c:v>0.74</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2071,7 +2144,7 @@
                   <c:v>RTX 4090 DX11 URP</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>RTX 4090 DX12  URP</c:v>
+                  <c:v>RTX 4090 DX12 URP</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2089,10 +2162,10 @@
                   <c:v>863</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>864.2</c:v>
+                  <c:v>1028.7</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>610.4</c:v>
+                  <c:v>723.1</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2405,6 +2478,25 @@
             <c:bubble3D val="0"/>
             <c:spPr>
               <a:solidFill>
+                <a:schemeClr val="accent1"/>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-46AB-46A9-B22D-022A5ACFB0FC}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
                 <a:schemeClr val="accent2"/>
               </a:solidFill>
               <a:ln>
@@ -2414,7 +2506,7 @@
             </c:spPr>
             <c:extLst>
               <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-                <c16:uniqueId val="{00000001-46AB-46A9-B22D-022A5ACFB0FC}"/>
+                <c16:uniqueId val="{00000002-40E6-4F11-AA65-8C21F84074FC}"/>
               </c:ext>
             </c:extLst>
           </c:dPt>
@@ -2451,10 +2543,10 @@
                   <c:v>9.66</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>9.5</c:v>
+                  <c:v>8.5299999999999994</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>11.98</c:v>
+                  <c:v>12.14</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -2783,7 +2875,7 @@
                   <c:v>RTX 4090 DX11 URP</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>RTX 4090 DX12  URP</c:v>
+                  <c:v>RTX 4090 DX12 URP</c:v>
                 </c:pt>
               </c:strCache>
             </c:strRef>
@@ -2801,10 +2893,10 @@
                   <c:v>1.1599999999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>1.1599999999999999</c:v>
+                  <c:v>0.97</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.64</c:v>
+                  <c:v>1.38</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -8875,48 +8967,48 @@
         <v>4</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="H2" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="I2" s="4" t="s">
         <v>3</v>
       </c>
       <c r="L2" s="4" t="s">
+        <v>9</v>
+      </c>
+      <c r="M2" s="4" t="s">
         <v>10</v>
-      </c>
-      <c r="M2" s="4" t="s">
-        <v>11</v>
       </c>
       <c r="N2" s="4" t="s">
         <v>1</v>
       </c>
       <c r="O2" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="P2" s="4" t="s">
         <v>3</v>
       </c>
       <c r="Q2" s="1"/>
       <c r="R2" s="4" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="S2" s="5"/>
       <c r="T2" s="4" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="U2" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="W2" s="4" t="s">
         <v>4</v>
       </c>
       <c r="X2" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3" spans="3:24" x14ac:dyDescent="0.35">
@@ -8924,7 +9016,7 @@
         <v>0</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E3" s="2" t="s">
         <v>5</v>
@@ -8962,7 +9054,7 @@
         <v>114</v>
       </c>
       <c r="R3" s="2" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="S3" s="2"/>
       <c r="T3" s="2">
@@ -8982,7 +9074,7 @@
         <v>0</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>5</v>
@@ -9020,16 +9112,16 @@
         <v>103.5</v>
       </c>
       <c r="R4" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="S4" s="2"/>
       <c r="T4" s="2">
         <f>H6</f>
-        <v>11.98</v>
+        <v>12.14</v>
       </c>
       <c r="U4" s="3">
         <f>(T4-T3)/T3</f>
-        <v>0.36602052451539352</v>
+        <v>0.38426453819840378</v>
       </c>
       <c r="W4" s="2" t="s">
         <v>6</v>
@@ -9043,22 +9135,22 @@
         <v>0</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F5" s="2">
-        <v>9.42</v>
+        <v>8.41</v>
       </c>
       <c r="G5" s="2">
-        <v>5.13</v>
+        <v>4.42</v>
       </c>
       <c r="H5" s="2">
-        <v>9.5</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="I5" s="2">
-        <v>105.3</v>
+        <v>117.2</v>
       </c>
       <c r="L5" s="2" t="str">
         <f t="shared" si="0"/>
@@ -9066,22 +9158,22 @@
       </c>
       <c r="M5" s="2">
         <f t="shared" si="1"/>
-        <v>9.42</v>
+        <v>8.41</v>
       </c>
       <c r="N5" s="2">
         <f t="shared" si="2"/>
-        <v>5.13</v>
+        <v>4.42</v>
       </c>
       <c r="O5" s="2">
         <f t="shared" si="3"/>
-        <v>9.5</v>
+        <v>8.5299999999999994</v>
       </c>
       <c r="P5" s="2">
         <f t="shared" si="4"/>
-        <v>105.3</v>
+        <v>117.2</v>
       </c>
       <c r="R5" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="S5" s="2"/>
       <c r="T5" s="2">
@@ -9095,22 +9187,22 @@
         <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E6" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F6" s="2">
-        <v>11.95</v>
+        <v>11.43</v>
       </c>
       <c r="G6" s="2">
-        <v>5.66</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="H6" s="2">
-        <v>11.98</v>
+        <v>12.14</v>
       </c>
       <c r="I6" s="2">
-        <v>83.5</v>
+        <v>82.4</v>
       </c>
       <c r="L6" s="2" t="str">
         <f t="shared" si="0"/>
@@ -9118,31 +9210,31 @@
       </c>
       <c r="M6" s="2">
         <f t="shared" si="1"/>
-        <v>11.95</v>
+        <v>11.43</v>
       </c>
       <c r="N6" s="2">
         <f t="shared" si="2"/>
-        <v>5.66</v>
+        <v>5.0999999999999996</v>
       </c>
       <c r="O6" s="2">
         <f t="shared" si="3"/>
-        <v>11.98</v>
+        <v>12.14</v>
       </c>
       <c r="P6" s="2">
         <f t="shared" si="4"/>
-        <v>83.5</v>
+        <v>82.4</v>
       </c>
       <c r="R6" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="S6" s="2"/>
       <c r="T6" s="2">
         <f>H10</f>
-        <v>1.64</v>
+        <v>1.38</v>
       </c>
       <c r="U6" s="3">
         <f>(T6-T5)/T5</f>
-        <v>1.0759493670886073</v>
+        <v>0.74683544303797444</v>
       </c>
     </row>
     <row r="7" spans="3:24" x14ac:dyDescent="0.35">
@@ -9150,7 +9242,7 @@
         <v>7</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E7" s="2" t="s">
         <v>5</v>
@@ -9193,7 +9285,7 @@
         <v>7</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>5</v>
@@ -9236,22 +9328,22 @@
         <v>7</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="E9" s="2" t="s">
         <v>6</v>
       </c>
       <c r="F9" s="2">
-        <v>1.1200000000000001</v>
+        <v>0.92</v>
       </c>
       <c r="G9" s="2">
-        <v>0.77</v>
+        <v>0.64</v>
       </c>
       <c r="H9" s="2">
-        <v>1.1599999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="I9" s="2">
-        <v>864.2</v>
+        <v>1028.7</v>
       </c>
       <c r="L9" s="2" t="str">
         <f t="shared" si="0"/>
@@ -9259,19 +9351,19 @@
       </c>
       <c r="M9" s="2">
         <f t="shared" si="1"/>
-        <v>1.1200000000000001</v>
+        <v>0.92</v>
       </c>
       <c r="N9" s="2">
         <f t="shared" si="2"/>
-        <v>0.77</v>
+        <v>0.64</v>
       </c>
       <c r="O9" s="2">
         <f t="shared" si="3"/>
-        <v>1.1599999999999999</v>
+        <v>0.97</v>
       </c>
       <c r="P9" s="2">
         <f t="shared" si="4"/>
-        <v>864.2</v>
+        <v>1028.7</v>
       </c>
     </row>
     <row r="10" spans="3:24" x14ac:dyDescent="0.35">
@@ -9279,42 +9371,42 @@
         <v>7</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="F10" s="2">
-        <v>1.61</v>
+        <v>1.36</v>
       </c>
       <c r="G10" s="2">
-        <v>0.83</v>
+        <v>0.74</v>
       </c>
       <c r="H10" s="2">
-        <v>1.64</v>
+        <v>1.38</v>
       </c>
       <c r="I10" s="2">
-        <v>610.4</v>
+        <v>723.1</v>
       </c>
       <c r="L10" s="2" t="str">
         <f t="shared" si="0"/>
-        <v>RTX 4090 DX12  URP</v>
+        <v>RTX 4090 DX12 URP</v>
       </c>
       <c r="M10" s="2">
         <f t="shared" si="1"/>
-        <v>1.61</v>
+        <v>1.36</v>
       </c>
       <c r="N10" s="2">
         <f t="shared" si="2"/>
-        <v>0.83</v>
+        <v>0.74</v>
       </c>
       <c r="O10" s="2">
         <f t="shared" si="3"/>
-        <v>1.64</v>
+        <v>1.38</v>
       </c>
       <c r="P10" s="2">
         <f t="shared" si="4"/>
-        <v>610.4</v>
+        <v>723.1</v>
       </c>
     </row>
   </sheetData>

</xml_diff>